<commit_message>
Add operators active in the stream for top 5 areas
New 'Top 5 Area Providers' workbook sheet + analysis/top5-area-providers.md:
2-4 registered providers / ALMOs / BTR operators delivering social & affordable
rent in Stoke-on-Trent, Hull & East Riding, Teesside, Wolverhampton/Black
Country and Doncaster. All verified via public/council sources.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134z6T1johUqsS5iLexF3Jz
</commit_message>
<xml_diff>
--- a/analysis/uk-rent-convergence-analysis.xlsx
+++ b/analysis/uk-rent-convergence-analysis.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Convergence Metric" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Verified Data Anchors" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Top 5 Area Providers" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,7 +49,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +64,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,6 +118,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2185,4 +2194,490 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="66" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Operators active in this revenue stream - Top 5 areas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Registered providers (RPs), council ALMOs and for-profit build-to-rent (BTR) operators currently delivering social &amp; affordable rent (incl. Affordable Rent at 80% of market) in each area. Most are not-for-profit RPs - the dominant operators of this stream. Verified via public/council sources (Sept 2024-2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Relevance to this revenue stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Stoke-on-Trent</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Aspire Housing</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>RP (housing association)</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>North Staffs/Stoke &amp; Newcastle-under-Lyme RP developing new affordable homes; in merger talks with whg (would create ~32,000-home Midlands group).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Stoke-on-Trent</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Honeycomb Group (incl. Staffs Housing)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>RP / charity</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Provides affordable housing and specialist support across Staffordshire, Cheshire and Derbyshire; Stoke-based.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Stoke-on-Trent</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Stoke-on-Trent Housing Society</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>RP (charitable HA)</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>621 homes across the city; actively builds new homes to meet local housing need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Stoke-on-Trent</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>EPIC Housing</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>RP (community HA)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>~1,400 homes at affordable rents across Stoke, Newcastle-under-Lyme and Staffordshire Moorlands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Kingston upon Hull &amp; East Riding</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Riverside</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>RP (large national HA)</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Dedicated Hull operations delivering social/affordable rent plus care &amp; support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Kingston upon Hull &amp; East Riding</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Pickering &amp; Ferens Homes (PFH)</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>RP (housing association)</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>~1,400 homes across Hull &amp; East Riding (predominantly older-persons affordable housing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Kingston upon Hull &amp; East Riding</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Hull Churches Housing Association</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>RP (independent HA)</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>~500 homes for social rent &amp; shared ownership in Hull and adjoining East Riding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Kingston upon Hull &amp; East Riding</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Sanctuary</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>RP (large national HA)</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>National RP with a Hull office/presence providing affordable rented homes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Teesside (Middlesbrough/Stockton/Redcar)</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Thirteen Group</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>RP (housing association)</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Teesside-based; ~34,000 homes mostly in Teesside - the largest local social landlord and an active developer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Teesside (Middlesbrough/Stockton/Redcar)</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Beyond Housing</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>RP (housing association)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Major RP across Redcar &amp; Cleveland / Tees Valley; core partner in Tees Valley Homefinder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Teesside (Middlesbrough/Stockton/Redcar)</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>North Star Housing Group</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>RP (housing association)</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Stockton-based RP; core partner in Tees Valley Homefinder and the Tees Valley Housing Partnership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Teesside (Middlesbrough/Stockton/Redcar)</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>The PRS REIT</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>For-profit build-to-rent</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>For-profit single-family BTR active in Teesside - example of the commercial side of the same rented-housing stream.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Wolverhampton / Black Country</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>whg (Walsall Housing Group)</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>RP (large HA)</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Large Midlands RP (Walsall HQ) delivering new affordable/social homes (e.g. Royal Hospital site: 154 homes for affordable rent &amp; shared ownership).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Wolverhampton / Black Country</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Bromford</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>RP (large HA / developer)</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Wolverhampton-HQ RP; major West Midlands developer via the 'Homes for the West Midlands' partnership (100% affordable Black Country scheme).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Wolverhampton / Black Country</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Black Country Housing Group (BCHG)</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>RP (housing association)</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Black Country RP providing affordable rented homes and support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Wolverhampton / Black Country</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Wolverhampton Homes</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Council ALMO</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Arm's-length organisation managing the City of Wolverhampton Council's social rented stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Doncaster</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>St Leger Homes of Doncaster</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Council ALMO</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Manages ~20,000 homes for City of Doncaster Council - the dominant social landlord; runs the Choice Based Lettings scheme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Doncaster</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Together Housing</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>RP (large HA)</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Delivering new affordable homes in Doncaster (2024 scheme with Housing 21 as part of a diverse development).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Doncaster</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Housing 21</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>RP (older-persons HA)</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Retirement/older-persons RP partnering on affordable-homes delivery in Doncaster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Note: this maps who is active in the stream, not an endorsement or a claim of current tenders. RP = Registered Provider; ALMO = Arm's Length Management Organisation. Verify current pipeline/JV appetite directly before acting.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A25:D25"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add provider stock size and RSH grades to top-5 providers
Extend 'Top 5 Area Providers' sheet + markdown with homes-owned, RSH
governance/viability/consumer grades and development/merger notes.
Integrity markers: ~approx, n/v not verified, — not applicable (ALMO/small
RP/for-profit), * widely-reported figure. ALMOs and for-profit BTR flagged
as outside the standard G/V regime.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134z6T1johUqsS5iLexF3Jz
</commit_message>
<xml_diff>
--- a/analysis/uk-rent-convergence-analysis.xlsx
+++ b/analysis/uk-rent-convergence-analysis.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -120,6 +120,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2202,13 +2211,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="66" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2243,7 +2256,27 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Relevance to this revenue stream</t>
+          <t>Homes (approx)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Notes (relevance / RSH judgement / development)</t>
         </is>
       </c>
     </row>
@@ -2260,12 +2293,32 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>RP (housing association)</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>North Staffs/Stoke &amp; Newcastle-under-Lyme RP developing new affordable homes; in merger talks with whg (would create ~32,000-home Midlands group).</t>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>~9,300</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>North Staffs/Stoke &amp; Cheshire; developing new affordable homes; in merger talks with whg (~32,000-home group). RJ Nov 2025.</t>
         </is>
       </c>
     </row>
@@ -2285,9 +2338,29 @@
           <t>RP / charity</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Provides affordable housing and specialist support across Staffordshire, Cheshire and Derbyshire; Stoke-based.</t>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>~3,118</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Affordable housing &amp; support across Staffs, Cheshire, Derbyshire. RSH judgement Oct 2025 (grades not captured this pass).</t>
         </is>
       </c>
     </row>
@@ -2304,12 +2377,32 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>RP (charitable HA)</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>621 homes across the city; actively builds new homes to meet local housing need.</t>
+          <t>RP (charitable)</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>621</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Under 1,000 homes: not individually graded by RSH. Actively builds new homes in the city.</t>
         </is>
       </c>
     </row>
@@ -2326,12 +2419,32 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>RP (community HA)</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>~1,400 homes at affordable rents across Stoke, Newcastle-under-Lyme and Staffordshire Moorlands.</t>
+          <t>RP (community)</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>~1,400</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Affordable rents across Stoke, Newcastle-under-Lyme and Staffordshire Moorlands.</t>
         </is>
       </c>
     </row>
@@ -2348,12 +2461,32 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>RP (large national HA)</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Dedicated Hull operations delivering social/affordable rent plus care &amp; support.</t>
+          <t>RP (large national)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>~75,000*</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Dedicated Hull operations (rent + care). RJ Mar 2024: G1 upgrade, V2 retained. *widely-reported total, confirm.</t>
         </is>
       </c>
     </row>
@@ -2370,12 +2503,32 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>RP (housing association)</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>~1,400 homes across Hull &amp; East Riding (predominantly older-persons affordable housing).</t>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>~1,400</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Older-persons affordable housing across Hull &amp; East Riding.</t>
         </is>
       </c>
     </row>
@@ -2392,12 +2545,32 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>RP (independent HA)</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>~500 homes for social rent &amp; shared ownership in Hull and adjoining East Riding.</t>
+          <t>RP (independent)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>~500</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Under 1,000 homes: not individually graded. Social rent &amp; shared ownership in Hull and adjoining East Riding.</t>
         </is>
       </c>
     </row>
@@ -2414,12 +2587,32 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>RP (large national HA)</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>National RP with a Hull office/presence providing affordable rented homes.</t>
+          <t>RP (large national)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>~120,000*</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Hull office/presence. C2 from planned inspection Jan 2025. *widely-reported total, confirm.</t>
         </is>
       </c>
     </row>
@@ -2436,12 +2629,32 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>RP (housing association)</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>Teesside-based; ~34,000 homes mostly in Teesside - the largest local social landlord and an active developer.</t>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>~34,000</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Teesside's largest social landlord and an active developer. C1 from inspection Mar 2025.</t>
         </is>
       </c>
     </row>
@@ -2458,12 +2671,32 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>RP (housing association)</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Major RP across Redcar &amp; Cleveland / Tees Valley; core partner in Tees Valley Homefinder.</t>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>~15,350</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Redcar/Tees Valley; core Tees Valley Homefinder partner. G1 upgrade Mar 2024.</t>
         </is>
       </c>
     </row>
@@ -2480,12 +2713,32 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>RP (housing association)</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Stockton-based RP; core partner in Tees Valley Homefinder and the Tees Valley Housing Partnership.</t>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>~4,000</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Stockton-based; Tees Valley partnership. RJ Dec 2024.</t>
         </is>
       </c>
     </row>
@@ -2502,12 +2755,32 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>For-profit build-to-rent</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>For-profit single-family BTR active in Teesside - example of the commercial side of the same rented-housing stream.</t>
+          <t>For-profit BTR</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>~5,000+ (n/v)</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>For-profit provider outside the standard G/V regime; single-family build-to-rent active in Teesside.</t>
         </is>
       </c>
     </row>
@@ -2524,12 +2797,32 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>RP (large HA)</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Large Midlands RP (Walsall HQ) delivering new affordable/social homes (e.g. Royal Hospital site: 154 homes for affordable rent &amp; shared ownership).</t>
+          <t>RP (large)</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>~21,000</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Walsall HQ. Royal Hospital scheme = 154 affordable-rent/shared-ownership homes; reports top grade after inspection.</t>
         </is>
       </c>
     </row>
@@ -2546,12 +2839,32 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>RP (large HA / developer)</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>Wolverhampton-HQ RP; major West Midlands developer via the 'Homes for the West Midlands' partnership (100% affordable Black Country scheme).</t>
+          <t>RP (large / developer)</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>~47,000</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Wolverhampton HQ; major developer ('Homes for the West Midlands'). LiveWest merger reported early 2026 - combined scale to confirm.</t>
         </is>
       </c>
     </row>
@@ -2568,10 +2881,30 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>RP (housing association)</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>&gt;2,000</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Black Country RP providing affordable rented homes and support.</t>
         </is>
@@ -2593,9 +2926,29 @@
           <t>Council ALMO</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Arm's-length organisation managing the City of Wolverhampton Council's social rented stock.</t>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>~21,000 (managed)</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Manages City of Wolverhampton Council stock; council holds the provider registration (not separately G/V graded); subject to consumer standards.</t>
         </is>
       </c>
     </row>
@@ -2615,9 +2968,29 @@
           <t>Council ALMO</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Manages ~20,000 homes for City of Doncaster Council - the dominant social landlord; runs the Choice Based Lettings scheme.</t>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>~20,000 (managed)</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>ALMO for City of Doncaster Council (council holds registration; subject to consumer standards). Runs Choice Based Lettings.</t>
         </is>
       </c>
     </row>
@@ -2634,12 +3007,32 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>RP (large HA)</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Delivering new affordable homes in Doncaster (2024 scheme with Housing 21 as part of a diverse development).</t>
+          <t>RP (large)</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>~36,000</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>n/v</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Delivering new affordable homes in Doncaster (2024 scheme with Housing 21). Viability regraded V1-&gt;V2.</t>
         </is>
       </c>
     </row>
@@ -2656,27 +3049,55 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>RP (older-persons HA)</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Retirement/older-persons RP partnering on affordable-homes delivery in Doncaster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
+          <t>RP (older-persons)</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>~23,300</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Retirement/ExtraCare across ~240 LAs; partnering on affordable-homes delivery in Doncaster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="56" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Legend: G=governance, V=viability, C=consumer (RSH grades; 1=strongest). n/v = not verified in this pass. — = not applicable (ALMO: the council holds the provider registration; or under-1,000-home RP not individually graded; or for-profit outside the G/V regime). * = widely-reported round figure, confirm. Grades change - re-check current RSH regulatory judgements before relying on them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Note: this maps who is active in the stream, not an endorsement or a claim of current tenders. RP = Registered Provider; ALMO = Arm's Length Management Organisation. Verify current pipeline/JV appetite directly before acting.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A24:H24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add measured convergence ranking from supplied ONS/LHA/RSH data
Real computation over the three supplied official datasets (97 LAs scored):
- run_measured_ranking.py + measured_convergence_ranking.csv
- MEASURED-RESULTS.md: findings, mechanism, how it revises the pattern list
- 'Measured Ranking' workbook sheet
- source files committed under analysis/data/ (OGL)

Thesis validated (all top-25 are low-cost North/Midlands; least-converged all
high-rent South). Order revised: East Lancs promoted, Black Country lowered on
pure convergence. Corrected Hull LHA to the authoritative DWP file
(87.45/109.32/126.58 pw), superseding an earlier web figure.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134z6T1johUqsS5iLexF3Jz
</commit_message>
<xml_diff>
--- a/analysis/uk-rent-convergence-analysis.xlsx
+++ b/analysis/uk-rent-convergence-analysis.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Verified Data Anchors" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Top 5 Area Providers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Measured Ranking" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -98,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +129,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -598,7 +602,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Sourced LHA close to market (1b GBP101.92 / 2b GBP126.92 / 3b GBP150.00 pw); tight 1-3 bed spread</t>
+          <t>Measured #5 of 97. LHA close to market (2-bed 474 vs 495/mo; align 0.96); tight 1-3 bed spread</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1622,7 +1626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1866,17 +1870,17 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>GBP 101.92 / wk (approx GBP 442/mo)</t>
+          <t>GBP 87.45 / wk (approx GBP 379/mo)</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>Apr-2024 base</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>VOA/council (6)</t>
+          <t>DWP/VOA LHA file (6)</t>
         </is>
       </c>
     </row>
@@ -1888,17 +1892,17 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>GBP 126.92 / wk (approx GBP 550/mo)</t>
+          <t>GBP 109.32 / wk (approx GBP 474/mo)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>Apr-2024 base</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>VOA/council (6)</t>
+          <t>DWP/VOA LHA file (6)</t>
         </is>
       </c>
     </row>
@@ -1910,56 +1914,56 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>GBP 150.00 / wk (approx GBP 650/mo)</t>
+          <t>GBP 126.58 / wk (approx GBP 549/mo)</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>Apr-2024 base</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>VOA/council (6)</t>
+          <t>DWP/VOA LHA file (6)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Households on LA housing registers</t>
+          <t>Hull market median (1/2/3 bed)</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>1.33 million (highest since 2014)</t>
+          <t>GBP 425 / 495 / 575 per month</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>31 Mar 2024</t>
+          <t>Oct22-Sep23</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>MHCLG (7)</t>
+          <t>ONS PRMS (supplied)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>London share of national register</t>
+          <t>Households on LA housing registers</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>approx 25%</t>
+          <t>1.33 million (highest since 2014)</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>31 Mar 2024</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -1971,20 +1975,42 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
+          <t>London share of national register</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>approx 25%</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>MHCLG (7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
           <t>Households in temporary accommodation</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>130,890 (+11.5% YoY)</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>31 Mar 2025</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>MHCLG (8)</t>
         </is>
@@ -3101,4 +3127,1536 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MEASURED convergence ranking (from supplied ONS + LHA + RSH data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="56" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Computed by run_measured_ranking.py. Market rent = ONS PRMS median by LA (Oct 2022-Sep 2023); LHA = DWP/VOA Apr-2024 base (monthly); social = England benchmark GBP113.69/wk (per-LA not supplied). Rents matched to the LHA base window = structural convergence, not today's live gap. geo: exact = name match, curated = our LA-&gt;BRMA map (dominant BRMA). 97 areas scored; top 30 shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Area (LA)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>BRMA</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Geo</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Sample</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Mkt 1b</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Mkt 2b</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Mkt 3b</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>LHA 2b</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Align</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>SocAtt</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Compr</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Burnley</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>East Lancs</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>420</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>475</v>
+      </c>
+      <c r="H5" s="13" t="n">
+        <v>550</v>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>474</v>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="13" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="M5" s="13" t="n">
+        <v>0.966</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Hartlepool UA</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Teesside</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>90</v>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>425</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>550</v>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>474</v>
+      </c>
+      <c r="J6" s="13" t="n">
+        <v>0.969</v>
+      </c>
+      <c r="K6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="13" t="n">
+        <v>0.896</v>
+      </c>
+      <c r="M6" s="13" t="n">
+        <v>0.956</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Hyndburn</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>East Lancs</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>425</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>495</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>600</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <v>474</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="K7" s="13" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="L7" s="13" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="M7" s="13" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>South Tyneside</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Tyneside</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>425</v>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>620</v>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>549</v>
+      </c>
+      <c r="J8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="13" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="L8" s="13" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="M8" s="13" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Kingston upon Hull, City of UA</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Hull &amp; East Riding</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>425</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>495</v>
+      </c>
+      <c r="H9" s="13" t="n">
+        <v>575</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>474</v>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>0.9340000000000001</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="L9" s="13" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="M9" s="13" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Pendle</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>East Lancs</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="G10" s="12" t="n">
+        <v>520</v>
+      </c>
+      <c r="H10" s="12" t="n">
+        <v>595</v>
+      </c>
+      <c r="I10" s="12" t="n">
+        <v>474</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>0.929</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>North East Lincolnshire UA</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Grimsby</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>420</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>525</v>
+      </c>
+      <c r="H11" s="12" t="n">
+        <v>565</v>
+      </c>
+      <c r="I11" s="12" t="n">
+        <v>479</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>0.879</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>0.927</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Rotherham</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Rotherham</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>475</v>
+      </c>
+      <c r="G12" s="12" t="n">
+        <v>550</v>
+      </c>
+      <c r="H12" s="12" t="n">
+        <v>570</v>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>499</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>0.924</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>0.924</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Redcar and Cleveland UA</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Teesside</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>438</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>510</v>
+      </c>
+      <c r="H13" s="12" t="n">
+        <v>593</v>
+      </c>
+      <c r="I13" s="12" t="n">
+        <v>474</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="K13" s="12" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="M13" s="12" t="n">
+        <v>0.922</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>County Durham UA</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Durham</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>260</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>380</v>
+      </c>
+      <c r="G14" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="H14" s="12" t="n">
+        <v>550</v>
+      </c>
+      <c r="I14" s="12" t="n">
+        <v>399</v>
+      </c>
+      <c r="J14" s="12" t="n">
+        <v>0.916</v>
+      </c>
+      <c r="K14" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="M14" s="12" t="n">
+        <v>0.921</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>North Lincolnshire UA</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Scunthorpe</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>433</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>525</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>607</v>
+      </c>
+      <c r="I15" s="12" t="n">
+        <v>494</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>0.864</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Gateshead</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Tyneside</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>110</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>475</v>
+      </c>
+      <c r="G16" s="12" t="n">
+        <v>580</v>
+      </c>
+      <c r="H16" s="12" t="n">
+        <v>650</v>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>549</v>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.873</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>0.914</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Blackburn with Darwen UA</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>East Lancs</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="F17" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="G17" s="12" t="n">
+        <v>524</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>620</v>
+      </c>
+      <c r="I17" s="12" t="n">
+        <v>474</v>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>0.9340000000000001</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>0.913</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Middlesbrough UA</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Teesside</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>525</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>595</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>474</v>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>0.911</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>0.913</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Blackpool UA</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Fylde Coast</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>430</v>
+      </c>
+      <c r="F19" s="12" t="n">
+        <v>412</v>
+      </c>
+      <c r="G19" s="12" t="n">
+        <v>550</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>650</v>
+      </c>
+      <c r="I19" s="12" t="n">
+        <v>540</v>
+      </c>
+      <c r="J19" s="12" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="K19" s="12" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="L19" s="12" t="n">
+        <v>0.8179999999999999</v>
+      </c>
+      <c r="M19" s="12" t="n">
+        <v>0.909</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Stoke-on-Trent UA</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Staffordshire North</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="G20" s="12" t="n">
+        <v>515</v>
+      </c>
+      <c r="H20" s="12" t="n">
+        <v>636</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>479</v>
+      </c>
+      <c r="J20" s="12" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="K20" s="12" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>0.856</v>
+      </c>
+      <c r="M20" s="12" t="n">
+        <v>0.908</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Doncaster</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Doncaster</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>320</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>475</v>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>550</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>600</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>499</v>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>0.904</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>0.906</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Darlington UA</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Darlington</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>270</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>605</v>
+      </c>
+      <c r="I22" s="12" t="n">
+        <v>449</v>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Barnsley</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Barnsley</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="n">
+        <v>190</v>
+      </c>
+      <c r="F23" s="12" t="n">
+        <v>475</v>
+      </c>
+      <c r="G23" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="H23" s="12" t="n">
+        <v>625</v>
+      </c>
+      <c r="I23" s="12" t="n">
+        <v>449</v>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>0.924</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>0.893</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Sunderland</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Sunderland</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="n">
+        <v>140</v>
+      </c>
+      <c r="F24" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="G24" s="12" t="n">
+        <v>550</v>
+      </c>
+      <c r="H24" s="12" t="n">
+        <v>625</v>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>474</v>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <v>0.891</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Preston</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Central Lancs</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="n">
+        <v>210</v>
+      </c>
+      <c r="F25" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="G25" s="12" t="n">
+        <v>600</v>
+      </c>
+      <c r="H25" s="12" t="n">
+        <v>675</v>
+      </c>
+      <c r="I25" s="12" t="n">
+        <v>573</v>
+      </c>
+      <c r="J25" s="12" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="K25" s="12" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="L25" s="12" t="n">
+        <v>0.879</v>
+      </c>
+      <c r="M25" s="12" t="n">
+        <v>0.889</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Northumberland UA</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Northumberland</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="F26" s="12" t="n">
+        <v>425</v>
+      </c>
+      <c r="G26" s="12" t="n">
+        <v>495</v>
+      </c>
+      <c r="H26" s="12" t="n">
+        <v>616</v>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>424</v>
+      </c>
+      <c r="J26" s="12" t="n">
+        <v>0.865</v>
+      </c>
+      <c r="K26" s="12" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="L26" s="12" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="M26" s="12" t="n">
+        <v>0.888</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Barrow-in-Furness</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Barrow-in-Furness</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>495</v>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>550</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>695</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>499</v>
+      </c>
+      <c r="J27" s="12" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="K27" s="12" t="n">
+        <v>0.849</v>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="M27" s="12" t="n">
+        <v>0.881</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>North Tyneside</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Tyneside</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>160</v>
+      </c>
+      <c r="F28" s="12" t="n">
+        <v>475</v>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>575</v>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>725</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>549</v>
+      </c>
+      <c r="J28" s="12" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="K28" s="12" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="M28" s="12" t="n">
+        <v>0.877</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Lancaster</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Lancaster</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>290</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>525</v>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>600</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>705</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>573</v>
+      </c>
+      <c r="J29" s="12" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="K29" s="12" t="n">
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>0.879</v>
+      </c>
+      <c r="M29" s="12" t="n">
+        <v>0.876</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Stockton-on-Tees UA</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Teesside</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="n">
+        <v>180</v>
+      </c>
+      <c r="F30" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="G30" s="12" t="n">
+        <v>550</v>
+      </c>
+      <c r="H30" s="12" t="n">
+        <v>650</v>
+      </c>
+      <c r="I30" s="12" t="n">
+        <v>474</v>
+      </c>
+      <c r="J30" s="12" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="K30" s="12" t="n">
+        <v>0.896</v>
+      </c>
+      <c r="L30" s="12" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="M30" s="12" t="n">
+        <v>0.873</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Scarborough</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Scarborough</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="n">
+        <v>180</v>
+      </c>
+      <c r="F31" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="G31" s="12" t="n">
+        <v>600</v>
+      </c>
+      <c r="H31" s="12" t="n">
+        <v>700</v>
+      </c>
+      <c r="I31" s="12" t="n">
+        <v>549</v>
+      </c>
+      <c r="J31" s="12" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="K31" s="12" t="n">
+        <v>0.845</v>
+      </c>
+      <c r="L31" s="12" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="M31" s="12" t="n">
+        <v>0.871</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Calderdale</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Halifax</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="F32" s="12" t="n">
+        <v>488</v>
+      </c>
+      <c r="G32" s="12" t="n">
+        <v>575</v>
+      </c>
+      <c r="H32" s="12" t="n">
+        <v>700</v>
+      </c>
+      <c r="I32" s="12" t="n">
+        <v>524</v>
+      </c>
+      <c r="J32" s="12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K32" s="12" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="L32" s="12" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="M32" s="12" t="n">
+        <v>0.867</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Wigan</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Wigan</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>290</v>
+      </c>
+      <c r="F33" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="G33" s="12" t="n">
+        <v>570</v>
+      </c>
+      <c r="H33" s="12" t="n">
+        <v>675</v>
+      </c>
+      <c r="I33" s="12" t="n">
+        <v>499</v>
+      </c>
+      <c r="J33" s="12" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="K33" s="12" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="L33" s="12" t="n">
+        <v>0.837</v>
+      </c>
+      <c r="M33" s="12" t="n">
+        <v>0.865</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Bradford</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Bradford &amp; South Dales</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="n">
+        <v>610</v>
+      </c>
+      <c r="F34" s="12" t="n">
+        <v>495</v>
+      </c>
+      <c r="G34" s="12" t="n">
+        <v>595</v>
+      </c>
+      <c r="H34" s="12" t="n">
+        <v>700</v>
+      </c>
+      <c r="I34" s="12" t="n">
+        <v>524</v>
+      </c>
+      <c r="J34" s="12" t="n">
+        <v>0.897</v>
+      </c>
+      <c r="K34" s="12" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="L34" s="12" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="M34" s="12" t="n">
+        <v>0.864</v>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Full 97-area table: analysis/measured_convergence_ranking.csv. See MEASURED-RESULTS.md for interpretation, the social-rent caveat, and how this revises the pattern-based ranking (e.g. East Lancs promoted, Black Country lowered on pure convergence).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A35:M35"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Use real per-LA social rents in measured ranking
Integrate RSH combined tool (Flat_File): per-LA, per-bedsize general-needs
social rent, weighted PRP+LARP, joined on ONS area E-code. 92/97 areas now use
local social rent (5 national fallback). All three rent layers now local; only
LA->BRMA geography is curated.

Result refined: Teesside rises to the top convergence cluster (Hartlepool #2,
Redcar #3, Middlesbrough #5); Hull eases to #12 (its social rents are among the
lowest nationally). Updated MEASURED-RESULTS.md, report Hull anchor, and the
workbook Measured Ranking sheet (now shows local social rent). Shadow List of
Rents file noted as LHA-basis data, not the geography lookup, so not used.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134z6T1johUqsS5iLexF3Jz
</commit_message>
<xml_diff>
--- a/analysis/uk-rent-convergence-analysis.xlsx
+++ b/analysis/uk-rent-convergence-analysis.xlsx
@@ -3163,7 +3163,7 @@
     <row r="2" ht="56" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Computed by run_measured_ranking.py. Market rent = ONS PRMS median by LA (Oct 2022-Sep 2023); LHA = DWP/VOA Apr-2024 base (monthly); social = England benchmark GBP113.69/wk (per-LA not supplied). Rents matched to the LHA base window = structural convergence, not today's live gap. geo: exact = name match, curated = our LA-&gt;BRMA map (dominant BRMA). 97 areas scored; top 30 shown.</t>
+          <t>Computed by run_measured_ranking.py. Market = ONS PRMS median by LA (Oct 2022-Sep 2023); LHA = DWP/VOA Apr-2024 base (monthly); social = RSH 2024/25 LOCAL per-bed general-needs rent (92/97 areas; 5 national fallback). Rents matched to the LHA base window = structural convergence, not today's live gap. geo: exact = name match, curated = our LA-&gt;BRMA map. 97 areas; top 30 shown.</t>
         </is>
       </c>
     </row>
@@ -3190,14 +3190,14 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>Soc src</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>Sample</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Mkt 1b</t>
-        </is>
-      </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Mkt 2b</t>
@@ -3205,12 +3205,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Mkt 3b</t>
+          <t>LHA 2b</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>LHA 2b</t>
+          <t>Soc 2b</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -3253,32 +3253,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="n">
         <v>40</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>420</v>
       </c>
       <c r="G5" s="13" t="n">
         <v>475</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>550</v>
+        <v>474</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>474</v>
+        <v>425</v>
       </c>
       <c r="J5" s="13" t="n">
         <v>0.999</v>
       </c>
       <c r="K5" s="13" t="n">
-        <v>1</v>
+        <v>0.872</v>
       </c>
       <c r="L5" s="13" t="n">
         <v>0.889</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>0.966</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="6">
@@ -3300,32 +3302,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="n">
         <v>90</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>425</v>
       </c>
       <c r="G6" s="13" t="n">
         <v>500</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>550</v>
+        <v>474</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>474</v>
+        <v>441</v>
       </c>
       <c r="J6" s="13" t="n">
         <v>0.969</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>1</v>
+        <v>0.882</v>
       </c>
       <c r="L6" s="13" t="n">
         <v>0.896</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>0.956</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="7">
@@ -3334,12 +3338,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Hyndburn</t>
+          <t>Redcar and Cleveland UA</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>East Lancs</t>
+          <t>Teesside</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -3347,32 +3351,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E7" s="13" t="n">
-        <v>70</v>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>425</v>
+        <v>130</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>495</v>
+        <v>510</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>600</v>
+        <v>474</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>474</v>
+        <v>461</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>0.981</v>
+        <v>0.929</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>0.972</v>
+        <v>0.903</v>
       </c>
       <c r="L7" s="13" t="n">
-        <v>0.858</v>
+        <v>0.877</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.906</v>
       </c>
     </row>
     <row r="8">
@@ -3381,12 +3387,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>South Tyneside</t>
+          <t>Hyndburn</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Tyneside</t>
+          <t>East Lancs</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -3394,32 +3400,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E8" s="13" t="n">
-        <v>50</v>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>425</v>
+        <v>70</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>620</v>
+        <v>474</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>549</v>
+        <v>403</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>1</v>
+        <v>0.981</v>
       </c>
       <c r="K8" s="13" t="n">
-        <v>0.957</v>
+        <v>0.798</v>
       </c>
       <c r="L8" s="13" t="n">
-        <v>0.844</v>
+        <v>0.858</v>
       </c>
       <c r="M8" s="13" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.889</v>
       </c>
     </row>
     <row r="9">
@@ -3428,12 +3436,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Kingston upon Hull, City of UA</t>
+          <t>Middlesbrough UA</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Hull &amp; East Riding</t>
+          <t>Teesside</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
@@ -3441,32 +3449,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E9" s="13" t="n">
-        <v>400</v>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>425</v>
+        <v>80</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>495</v>
+        <v>525</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>575</v>
+        <v>474</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>474</v>
+        <v>450</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.911</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>0.989</v>
+        <v>0.859</v>
       </c>
       <c r="L9" s="13" t="n">
-        <v>0.877</v>
+        <v>0.887</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.888</v>
       </c>
     </row>
     <row r="10">
@@ -3475,45 +3485,47 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Pendle</t>
+          <t>Barrow-in-Furness</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>East Lancs</t>
+          <t>Barrow-in-Furness</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>curated</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="n">
-        <v>90</v>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>national</t>
+        </is>
       </c>
       <c r="F10" s="12" t="n">
-        <v>450</v>
+        <v>70</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>520</v>
+        <v>550</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>595</v>
+        <v>499</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>474</v>
+        <v>493</v>
       </c>
       <c r="J10" s="12" t="n">
-        <v>0.95</v>
+        <v>0.925</v>
       </c>
       <c r="K10" s="12" t="n">
-        <v>0.944</v>
+        <v>0.867</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>0.887</v>
+        <v>0.855</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>0.929</v>
+        <v>0.886</v>
       </c>
     </row>
     <row r="11">
@@ -3522,12 +3534,12 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>North East Lincolnshire UA</t>
+          <t>South Tyneside</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Grimsby</t>
+          <t>Tyneside</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -3535,32 +3547,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E11" s="12" t="n">
-        <v>80</v>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F11" s="12" t="n">
-        <v>420</v>
+        <v>50</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>525</v>
+        <v>500</v>
       </c>
       <c r="H11" s="12" t="n">
-        <v>565</v>
+        <v>549</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>479</v>
+        <v>396</v>
       </c>
       <c r="J11" s="12" t="n">
-        <v>0.923</v>
+        <v>1</v>
       </c>
       <c r="K11" s="12" t="n">
-        <v>0.979</v>
+        <v>0.766</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>0.879</v>
+        <v>0.844</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>0.927</v>
+        <v>0.883</v>
       </c>
     </row>
     <row r="12">
@@ -3569,45 +3583,47 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Rotherham</t>
+          <t>North East Lincolnshire UA</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Rotherham</t>
+          <t>Grimsby</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>150</v>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F12" s="12" t="n">
-        <v>475</v>
+        <v>80</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>550</v>
+        <v>525</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>570</v>
+        <v>479</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>499</v>
+        <v>426</v>
       </c>
       <c r="J12" s="12" t="n">
-        <v>0.924</v>
+        <v>0.923</v>
       </c>
       <c r="K12" s="12" t="n">
-        <v>0.927</v>
+        <v>0.835</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>0.923</v>
+        <v>0.879</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>0.924</v>
+        <v>0.883</v>
       </c>
     </row>
     <row r="13">
@@ -3616,12 +3632,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Redcar and Cleveland UA</t>
+          <t>North Lincolnshire UA</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Teesside</t>
+          <t>Scunthorpe</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -3629,32 +3645,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E13" s="12" t="n">
-        <v>130</v>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F13" s="12" t="n">
-        <v>438</v>
+        <v>170</v>
       </c>
       <c r="G13" s="12" t="n">
-        <v>510</v>
+        <v>525</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>593</v>
+        <v>494</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>474</v>
+        <v>421</v>
       </c>
       <c r="J13" s="12" t="n">
-        <v>0.929</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="K13" s="12" t="n">
-        <v>0.959</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>0.877</v>
+        <v>0.864</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>0.922</v>
+        <v>0.879</v>
       </c>
     </row>
     <row r="14">
@@ -3663,12 +3681,12 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>County Durham UA</t>
+          <t>Pendle</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Durham</t>
+          <t>East Lancs</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
@@ -3676,32 +3694,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E14" s="12" t="n">
-        <v>260</v>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F14" s="12" t="n">
-        <v>380</v>
+        <v>90</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>550</v>
+        <v>474</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="J14" s="12" t="n">
-        <v>0.916</v>
+        <v>0.95</v>
       </c>
       <c r="K14" s="12" t="n">
-        <v>1</v>
+        <v>0.776</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>0.848</v>
+        <v>0.887</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>0.921</v>
+        <v>0.879</v>
       </c>
     </row>
     <row r="15">
@@ -3710,12 +3730,12 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>North Lincolnshire UA</t>
+          <t>County Durham UA</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Scunthorpe</t>
+          <t>Durham</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -3723,32 +3743,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E15" s="12" t="n">
-        <v>170</v>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F15" s="12" t="n">
-        <v>433</v>
+        <v>260</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>525</v>
+        <v>450</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>607</v>
+        <v>399</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>494</v>
+        <v>390</v>
       </c>
       <c r="J15" s="12" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.916</v>
       </c>
       <c r="K15" s="12" t="n">
-        <v>0.944</v>
+        <v>0.847</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>0.864</v>
+        <v>0.848</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>0.92</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="16">
@@ -3757,12 +3779,12 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Gateshead</t>
+          <t>Kingston upon Hull, City of UA</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Tyneside</t>
+          <t>Hull &amp; East Riding</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -3770,32 +3792,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E16" s="12" t="n">
-        <v>110</v>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F16" s="12" t="n">
-        <v>475</v>
+        <v>400</v>
       </c>
       <c r="G16" s="12" t="n">
-        <v>580</v>
+        <v>495</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>650</v>
+        <v>474</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>549</v>
+        <v>407</v>
       </c>
       <c r="J16" s="12" t="n">
-        <v>0.981</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>0.867</v>
+        <v>0.795</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>0.873</v>
+        <v>0.877</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>0.914</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="17">
@@ -3804,45 +3828,47 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Blackburn with Darwen UA</t>
+          <t>Rotherham</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>East Lancs</t>
+          <t>Rotherham</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>curated</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="n">
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="n">
         <v>150</v>
       </c>
-      <c r="F17" s="12" t="n">
-        <v>450</v>
-      </c>
       <c r="G17" s="12" t="n">
-        <v>524</v>
+        <v>550</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>620</v>
+        <v>499</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>474</v>
+        <v>401</v>
       </c>
       <c r="J17" s="12" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.924</v>
       </c>
       <c r="K17" s="12" t="n">
-        <v>0.927</v>
+        <v>0.75</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>0.869</v>
+        <v>0.923</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>0.913</v>
+        <v>0.872</v>
       </c>
     </row>
     <row r="18">
@@ -3851,45 +3877,47 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Middlesbrough UA</t>
+          <t>Scarborough</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Teesside</t>
+          <t>Scarborough</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>curated</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="n">
-        <v>80</v>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>national</t>
+        </is>
       </c>
       <c r="F18" s="12" t="n">
-        <v>450</v>
+        <v>180</v>
       </c>
       <c r="G18" s="12" t="n">
-        <v>525</v>
+        <v>600</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>595</v>
+        <v>549</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>474</v>
+        <v>493</v>
       </c>
       <c r="J18" s="12" t="n">
-        <v>0.911</v>
+        <v>0.927</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.842</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>0.887</v>
+        <v>0.824</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>0.913</v>
+        <v>0.871</v>
       </c>
     </row>
     <row r="19">
@@ -3898,12 +3926,12 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Blackpool UA</t>
+          <t>Gateshead</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Fylde Coast</t>
+          <t>Tyneside</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -3911,32 +3939,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E19" s="12" t="n">
-        <v>430</v>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F19" s="12" t="n">
-        <v>412</v>
+        <v>110</v>
       </c>
       <c r="G19" s="12" t="n">
-        <v>550</v>
+        <v>580</v>
       </c>
       <c r="H19" s="12" t="n">
-        <v>650</v>
+        <v>549</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>540</v>
+        <v>406</v>
       </c>
       <c r="J19" s="12" t="n">
-        <v>0.97</v>
+        <v>0.981</v>
       </c>
       <c r="K19" s="12" t="n">
-        <v>0.917</v>
+        <v>0.716</v>
       </c>
       <c r="L19" s="12" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.873</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>0.909</v>
+        <v>0.869</v>
       </c>
     </row>
     <row r="20">
@@ -3945,12 +3975,12 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Stoke-on-Trent UA</t>
+          <t>Blackburn with Darwen UA</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Staffordshire North</t>
+          <t>East Lancs</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -3958,32 +3988,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E20" s="12" t="n">
-        <v>200</v>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F20" s="12" t="n">
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="G20" s="12" t="n">
-        <v>515</v>
+        <v>524</v>
       </c>
       <c r="H20" s="12" t="n">
-        <v>636</v>
+        <v>474</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>479</v>
+        <v>412</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.923</v>
+        <v>0.776</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>0.856</v>
+        <v>0.869</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>0.908</v>
+        <v>0.867</v>
       </c>
     </row>
     <row r="21">
@@ -3992,45 +4024,47 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Doncaster</t>
+          <t>Blackpool UA</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Doncaster</t>
+          <t>Fylde Coast</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="E21" s="12" t="n">
-        <v>320</v>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F21" s="12" t="n">
-        <v>475</v>
+        <v>430</v>
       </c>
       <c r="G21" s="12" t="n">
         <v>550</v>
       </c>
       <c r="H21" s="12" t="n">
-        <v>600</v>
+        <v>540</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>499</v>
+        <v>404</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>0.904</v>
+        <v>0.97</v>
       </c>
       <c r="K21" s="12" t="n">
-        <v>0.91</v>
+        <v>0.748</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>0.905</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>0.906</v>
+        <v>0.858</v>
       </c>
     </row>
     <row r="22">
@@ -4039,12 +4073,12 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Darlington UA</t>
+          <t>Preston</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Darlington</t>
+          <t>Central Lancs</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -4052,32 +4086,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E22" s="12" t="n">
-        <v>270</v>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F22" s="12" t="n">
-        <v>400</v>
+        <v>210</v>
       </c>
       <c r="G22" s="12" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="H22" s="12" t="n">
-        <v>605</v>
+        <v>573</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>449</v>
+        <v>422</v>
       </c>
       <c r="J22" s="12" t="n">
-        <v>0.89</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="K22" s="12" t="n">
-        <v>0.982</v>
+        <v>0.705</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>0.833</v>
+        <v>0.879</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="23">
@@ -4086,45 +4122,47 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Barnsley</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Barnsley</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="E23" s="12" t="n">
-        <v>190</v>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F23" s="12" t="n">
-        <v>475</v>
+        <v>140</v>
       </c>
       <c r="G23" s="12" t="n">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>625</v>
+        <v>474</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>449</v>
+        <v>418</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>0.882</v>
+        <v>0.894</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>0.924</v>
+        <v>0.773</v>
       </c>
       <c r="L23" s="12" t="n">
-        <v>0.877</v>
+        <v>0.868</v>
       </c>
       <c r="M23" s="12" t="n">
-        <v>0.893</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="24">
@@ -4133,12 +4171,12 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Stoke-on-Trent UA</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Staffordshire North</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -4146,32 +4184,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E24" s="12" t="n">
-        <v>140</v>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F24" s="12" t="n">
-        <v>450</v>
+        <v>200</v>
       </c>
       <c r="G24" s="12" t="n">
-        <v>550</v>
+        <v>515</v>
       </c>
       <c r="H24" s="12" t="n">
-        <v>625</v>
+        <v>479</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>474</v>
+        <v>380</v>
       </c>
       <c r="J24" s="12" t="n">
-        <v>0.894</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="K24" s="12" t="n">
-        <v>0.91</v>
+        <v>0.717</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>0.868</v>
+        <v>0.856</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>0.891</v>
+        <v>0.846</v>
       </c>
     </row>
     <row r="25">
@@ -4180,12 +4220,12 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Stockton-on-Tees UA</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Central Lancs</t>
+          <t>Teesside</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
@@ -4193,32 +4233,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E25" s="12" t="n">
-        <v>210</v>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F25" s="12" t="n">
-        <v>500</v>
+        <v>180</v>
       </c>
       <c r="G25" s="12" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="H25" s="12" t="n">
-        <v>675</v>
+        <v>474</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>573</v>
+        <v>442</v>
       </c>
       <c r="J25" s="12" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.871</v>
       </c>
       <c r="K25" s="12" t="n">
-        <v>0.833</v>
+        <v>0.806</v>
       </c>
       <c r="L25" s="12" t="n">
-        <v>0.879</v>
+        <v>0.852</v>
       </c>
       <c r="M25" s="12" t="n">
-        <v>0.889</v>
+        <v>0.846</v>
       </c>
     </row>
     <row r="26">
@@ -4227,45 +4269,47 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Northumberland UA</t>
+          <t>Doncaster</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Northumberland</t>
+          <t>Doncaster</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>curated</t>
-        </is>
-      </c>
-      <c r="E26" s="12" t="n">
-        <v>150</v>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F26" s="12" t="n">
-        <v>425</v>
+        <v>320</v>
       </c>
       <c r="G26" s="12" t="n">
-        <v>495</v>
+        <v>550</v>
       </c>
       <c r="H26" s="12" t="n">
-        <v>616</v>
+        <v>499</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>424</v>
+        <v>384</v>
       </c>
       <c r="J26" s="12" t="n">
-        <v>0.865</v>
+        <v>0.904</v>
       </c>
       <c r="K26" s="12" t="n">
-        <v>0.962</v>
+        <v>0.702</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>0.846</v>
+        <v>0.905</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>0.888</v>
+        <v>0.844</v>
       </c>
     </row>
     <row r="27">
@@ -4274,12 +4318,12 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Barrow-in-Furness</t>
+          <t>St. Helens</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Barrow-in-Furness</t>
+          <t>St Helens</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -4287,32 +4331,34 @@
           <t>exact</t>
         </is>
       </c>
-      <c r="E27" s="12" t="n">
-        <v>70</v>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F27" s="12" t="n">
-        <v>495</v>
+        <v>110</v>
       </c>
       <c r="G27" s="12" t="n">
-        <v>550</v>
+        <v>575</v>
       </c>
       <c r="H27" s="12" t="n">
-        <v>695</v>
+        <v>524</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>499</v>
+        <v>451</v>
       </c>
       <c r="J27" s="12" t="n">
-        <v>0.925</v>
+        <v>0.886</v>
       </c>
       <c r="K27" s="12" t="n">
-        <v>0.849</v>
+        <v>0.769</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>0.855</v>
+        <v>0.857</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>0.881</v>
+        <v>0.842</v>
       </c>
     </row>
     <row r="28">
@@ -4321,45 +4367,47 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>North Tyneside</t>
+          <t>Barnsley</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Tyneside</t>
+          <t>Barnsley</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>curated</t>
-        </is>
-      </c>
-      <c r="E28" s="12" t="n">
-        <v>160</v>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F28" s="12" t="n">
-        <v>475</v>
+        <v>190</v>
       </c>
       <c r="G28" s="12" t="n">
-        <v>575</v>
+        <v>500</v>
       </c>
       <c r="H28" s="12" t="n">
-        <v>725</v>
+        <v>449</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>549</v>
+        <v>400</v>
       </c>
       <c r="J28" s="12" t="n">
-        <v>0.949</v>
+        <v>0.882</v>
       </c>
       <c r="K28" s="12" t="n">
-        <v>0.833</v>
+        <v>0.739</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>0.826</v>
+        <v>0.877</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>0.877</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="29">
@@ -4368,45 +4416,47 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Lancaster</t>
+          <t>Calderdale</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Lancaster</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="n">
-        <v>290</v>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F29" s="12" t="n">
-        <v>525</v>
+        <v>300</v>
       </c>
       <c r="G29" s="12" t="n">
-        <v>600</v>
+        <v>575</v>
       </c>
       <c r="H29" s="12" t="n">
-        <v>705</v>
+        <v>524</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>573</v>
+        <v>429</v>
       </c>
       <c r="J29" s="12" t="n">
-        <v>0.926</v>
+        <v>0.9</v>
       </c>
       <c r="K29" s="12" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.73</v>
       </c>
       <c r="L29" s="12" t="n">
-        <v>0.879</v>
+        <v>0.852</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>0.876</v>
+        <v>0.835</v>
       </c>
     </row>
     <row r="30">
@@ -4415,12 +4465,12 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Stockton-on-Tees UA</t>
+          <t>North Tyneside</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Teesside</t>
+          <t>Tyneside</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -4428,32 +4478,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E30" s="12" t="n">
-        <v>180</v>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F30" s="12" t="n">
-        <v>450</v>
+        <v>160</v>
       </c>
       <c r="G30" s="12" t="n">
-        <v>550</v>
+        <v>575</v>
       </c>
       <c r="H30" s="12" t="n">
-        <v>650</v>
+        <v>549</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>474</v>
+        <v>406</v>
       </c>
       <c r="J30" s="12" t="n">
-        <v>0.871</v>
+        <v>0.949</v>
       </c>
       <c r="K30" s="12" t="n">
-        <v>0.896</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>0.852</v>
+        <v>0.826</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>0.873</v>
+        <v>0.835</v>
       </c>
     </row>
     <row r="31">
@@ -4462,45 +4514,47 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Scarborough</t>
+          <t>Darlington UA</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Scarborough</t>
+          <t>Darlington</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="n">
-        <v>180</v>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F31" s="12" t="n">
-        <v>450</v>
+        <v>270</v>
       </c>
       <c r="G31" s="12" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="H31" s="12" t="n">
-        <v>700</v>
+        <v>449</v>
       </c>
       <c r="I31" s="12" t="n">
-        <v>549</v>
+        <v>379</v>
       </c>
       <c r="J31" s="12" t="n">
-        <v>0.927</v>
+        <v>0.89</v>
       </c>
       <c r="K31" s="12" t="n">
-        <v>0.845</v>
+        <v>0.761</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>0.824</v>
+        <v>0.833</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>0.871</v>
+        <v>0.834</v>
       </c>
     </row>
     <row r="32">
@@ -4509,45 +4563,47 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Calderdale</t>
+          <t>Lancaster</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Lancaster</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>curated</t>
-        </is>
-      </c>
-      <c r="E32" s="12" t="n">
-        <v>300</v>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F32" s="12" t="n">
-        <v>488</v>
+        <v>290</v>
       </c>
       <c r="G32" s="12" t="n">
-        <v>575</v>
+        <v>600</v>
       </c>
       <c r="H32" s="12" t="n">
-        <v>700</v>
+        <v>573</v>
       </c>
       <c r="I32" s="12" t="n">
-        <v>524</v>
+        <v>405</v>
       </c>
       <c r="J32" s="12" t="n">
-        <v>0.9</v>
+        <v>0.926</v>
       </c>
       <c r="K32" s="12" t="n">
-        <v>0.838</v>
+        <v>0.667</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>0.852</v>
+        <v>0.879</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>0.867</v>
+        <v>0.834</v>
       </c>
     </row>
     <row r="33">
@@ -4556,45 +4612,47 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Wigan</t>
+          <t>Knowsley</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Wigan</t>
+          <t>Greater Liverpool</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="E33" s="12" t="n">
-        <v>290</v>
+          <t>curated</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F33" s="12" t="n">
-        <v>450</v>
+        <v>20</v>
       </c>
       <c r="G33" s="12" t="n">
-        <v>570</v>
+        <v>625</v>
       </c>
       <c r="H33" s="12" t="n">
-        <v>675</v>
+        <v>593</v>
       </c>
       <c r="I33" s="12" t="n">
-        <v>499</v>
+        <v>431</v>
       </c>
       <c r="J33" s="12" t="n">
-        <v>0.88</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="K33" s="12" t="n">
-        <v>0.872</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="L33" s="12" t="n">
         <v>0.837</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>0.865</v>
+        <v>0.833</v>
       </c>
     </row>
     <row r="34">
@@ -4603,12 +4661,12 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Bradford</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Bradford &amp; South Dales</t>
+          <t>Black Country</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -4616,32 +4674,34 @@
           <t>curated</t>
         </is>
       </c>
-      <c r="E34" s="12" t="n">
-        <v>610</v>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
       </c>
       <c r="F34" s="12" t="n">
-        <v>495</v>
+        <v>170</v>
       </c>
       <c r="G34" s="12" t="n">
-        <v>595</v>
+        <v>650</v>
       </c>
       <c r="H34" s="12" t="n">
-        <v>700</v>
+        <v>623</v>
       </c>
       <c r="I34" s="12" t="n">
-        <v>524</v>
+        <v>442</v>
       </c>
       <c r="J34" s="12" t="n">
-        <v>0.897</v>
+        <v>0.93</v>
       </c>
       <c r="K34" s="12" t="n">
-        <v>0.826</v>
+        <v>0.679</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>0.86</v>
+        <v>0.846</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>0.864</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="35" ht="42" customHeight="1">

</xml_diff>